<commit_message>
Nettoyage navettes : supprime ancien format lot02/lot03, retire FAC-2026-001 de lot01
lot01 conserve uniquement la feuille template "Feuille1" créée manuellement.
lot02 et lot03 seront recréés avec la nouvelle présentation (style Feuille1).

https://claude.ai/code/session_01KKDRDc2csvTnXfsCnXGCHi
</commit_message>
<xml_diff>
--- a/data/navettes_et_bons/lot01 Isolation_thermique PlatrOMATIC.xlsx
+++ b/data/navettes_et_bons/lot01 Isolation_thermique PlatrOMATIC.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Feuille1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="FAC-2026-001" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
@@ -24,8 +23,8 @@
     <numFmt numFmtId="167" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* \-??\ [$€-40C]_-;_-@_-"/>
     <numFmt numFmtId="168" formatCode="0\ %"/>
     <numFmt numFmtId="169" formatCode="#,##0.00\ [$€-40C];[RED]\-#,##0.00\ [$€-40C]"/>
-    <numFmt numFmtId="170" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* \-??\ _€_-;_-@_-"/>
-    <numFmt numFmtId="171" formatCode="#,##0.00 &quot;EUR&quot;"/>
+    <numFmt numFmtId="170" formatCode="#,##0.00 &quot;EUR&quot;"/>
+    <numFmt numFmtId="171" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* \-??\ _€_-;_-@_-"/>
   </numFmts>
   <fonts count="46">
     <font>
@@ -615,7 +614,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="41" fontId="3" fillId="0" borderId="0"/>
@@ -1543,9 +1542,9 @@
       <alignment horizontal="general" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="171" fontId="45" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="45" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2991,240 +2990,4 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="38" customWidth="1" style="153" min="1" max="1"/>
-    <col width="22" customWidth="1" style="153" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="306" t="inlineStr">
-        <is>
-          <t>FICHE NAVETTE — PROJET renovation_2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MOE</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>RenovBat</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>MOA</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>IMMOSOCIAL_69</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Référence facture</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>FAC-2026-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Date de la facture</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>15 mars 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Émetteur</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Platr'O'Matic SARL</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Lot concerné</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>isolation_thermique</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Montant TTC</t>
-        </is>
-      </c>
-      <c r="B10" s="307" t="n">
-        <v>12500</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="308" t="inlineStr">
-        <is>
-          <t>✓ FACTURE APPROUVÉE</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Date d'approbation</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>24/04/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Approuvé par</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>RenovBat</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="306" t="inlineStr">
-        <is>
-          <t>BON DE PAIEMENT — PROJET renovation_2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Montant global prévu pour le lot</t>
-        </is>
-      </c>
-      <c r="B19" s="307" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Situations précédentes</t>
-        </is>
-      </c>
-      <c r="B20" s="307" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Présente situation</t>
-        </is>
-      </c>
-      <c r="B21" s="307" t="n">
-        <v>12500</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Nouveau cumul</t>
-        </is>
-      </c>
-      <c r="B23" s="309" t="n">
-        <v>12500</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Reste à régler</t>
-        </is>
-      </c>
-      <c r="B24" s="307" t="n">
-        <v>7500</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Date d'émission</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>24/04/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Établi par</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>RenovBat (MOE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>À destination de</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>IMMOSOCIAL_69 (MOA)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A12:B12"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>